<commit_message>
Implement till architecture v3
</commit_message>
<xml_diff>
--- a/resource/groundTruths/architecture/CF_M05_ground_truth_architecture.xlsx
+++ b/resource/groundTruths/architecture/CF_M05_ground_truth_architecture.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oguzarslan/Desktop/upc/semester-4/Thesis/MappingGenerator/resource/groundTruths/architecture/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{772D31A1-05A1-4C49-B449-6998EFECB5DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87B2446E-8CA3-0C4D-BDC9-4E98CCF422E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="16880" activeTab="1" xr2:uid="{6707339F-D318-8E46-9AE1-9A501C36040E}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="142">
   <si>
     <t>Document ID</t>
   </si>
@@ -439,9 +439,6 @@
     <t>Leader's main function is to route all communications to the corresponding microservice within the system architecture.</t>
   </si>
   <si>
-    <t>CF_M05_AU01, CF_M05_AU02, CF_M05_AU03, CF_M05_AU04, CF_M05_AU05, CF_M05_AU06, CF_M05_AU07</t>
-  </si>
-  <si>
     <t>Communication Log's main purpose is to record all communications that occur within the system, both between microservices and with external services.</t>
   </si>
   <si>
@@ -482,6 +479,37 @@
   </si>
   <si>
     <t>Fixed Type</t>
+  </si>
+  <si>
+    <t>On the other hand, the services are responsible for orchestrating HTTP calls to the server.</t>
+  </si>
+  <si>
+    <t>CF_M05_AU34</t>
+  </si>
+  <si>
+    <t>CF_M05_AU14, CF_M05_AU32</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
+    <t>64</t>
+  </si>
+  <si>
+    <t>CF_M05_AU04, CF_M05_AU01, CF_M05_AU02, CF_M05_AU03, CF_M05_AU05, CF_M05_AU06, CF_M05_AU07</t>
+  </si>
+  <si>
+    <t>CF_M05_AU35</t>
+  </si>
+  <si>
+    <t>Kubernetes</t>
+  </si>
+  <si>
+    <t>which allows the use of Kubernetes (K8s), a container orchestration platform created by
+Google, without the need to install or maintain it.</t>
+  </si>
+  <si>
+    <t>81</t>
   </si>
 </sst>
 </file>
@@ -599,7 +627,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -629,12 +657,6 @@
     <xf numFmtId="49" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -652,6 +674,16 @@
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -967,8 +999,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE9D1564-DBE6-2644-8A71-E3F0F3401448}">
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="7" max="7" width="10.83203125" style="19"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
@@ -989,11 +1024,11 @@
       <c r="F1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="20" t="s">
         <v>1</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
@@ -1003,19 +1038,19 @@
       <c r="B2" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="11" t="s">
         <v>21</v>
       </c>
       <c r="D2" t="s">
         <v>105</v>
       </c>
-      <c r="E2" s="14" t="s">
+      <c r="E2" s="12" t="s">
         <v>33</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="G2" s="11">
+      <c r="G2" s="17">
         <v>57</v>
       </c>
     </row>
@@ -1026,7 +1061,7 @@
       <c r="B3" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="11" t="s">
         <v>21</v>
       </c>
       <c r="D3" t="s">
@@ -1038,7 +1073,7 @@
       <c r="F3" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="G3" s="12">
+      <c r="G3" s="18">
         <v>57</v>
       </c>
     </row>
@@ -1049,19 +1084,19 @@
       <c r="B4" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="11" t="s">
         <v>21</v>
       </c>
       <c r="D4" t="s">
         <v>107</v>
       </c>
-      <c r="E4" s="14" t="s">
+      <c r="E4" s="12" t="s">
         <v>35</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="G4" s="11">
+      <c r="G4" s="17">
         <v>58</v>
       </c>
     </row>
@@ -1072,7 +1107,7 @@
       <c r="B5" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="11" t="s">
         <v>21</v>
       </c>
       <c r="D5" t="s">
@@ -1084,7 +1119,7 @@
       <c r="F5" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="G5" s="12">
+      <c r="G5" s="18">
         <v>58.59</v>
       </c>
     </row>
@@ -1095,19 +1130,19 @@
       <c r="B6" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="11" t="s">
         <v>21</v>
       </c>
       <c r="D6" t="s">
         <v>44</v>
       </c>
-      <c r="E6" s="14" t="s">
+      <c r="E6" s="12" t="s">
         <v>37</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="G6" s="11">
+      <c r="G6" s="17">
         <v>59.6</v>
       </c>
     </row>
@@ -1118,11 +1153,11 @@
       <c r="B7" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="C7" s="11" t="s">
         <v>19</v>
       </c>
       <c r="D7" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>20</v>
@@ -1130,7 +1165,7 @@
       <c r="F7" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="G7" s="12">
+      <c r="G7" s="18">
         <v>62</v>
       </c>
     </row>
@@ -1141,19 +1176,19 @@
       <c r="B8" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="11" t="s">
         <v>22</v>
       </c>
       <c r="D8" t="s">
         <v>43</v>
       </c>
-      <c r="E8" s="14" t="s">
+      <c r="E8" s="12" t="s">
         <v>38</v>
       </c>
       <c r="F8" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="G8" s="11">
+      <c r="G8" s="17">
         <v>81</v>
       </c>
     </row>
@@ -1164,7 +1199,7 @@
       <c r="B9" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="11" t="s">
         <v>22</v>
       </c>
       <c r="D9" t="s">
@@ -1173,10 +1208,10 @@
       <c r="E9" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="F9" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="G9" s="12">
+      <c r="G9" s="18">
         <v>84</v>
       </c>
     </row>
@@ -1187,7 +1222,7 @@
       <c r="B10" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="11" t="s">
         <v>22</v>
       </c>
       <c r="D10" t="s">
@@ -1196,10 +1231,10 @@
       <c r="E10" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="F10" s="13" t="s">
+      <c r="F10" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="G10" s="11">
+      <c r="G10" s="17">
         <v>87</v>
       </c>
     </row>
@@ -1207,10 +1242,10 @@
       <c r="A11" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="13" t="s">
+      <c r="B11" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="11" t="s">
         <v>22</v>
       </c>
       <c r="D11" t="s">
@@ -1222,7 +1257,7 @@
       <c r="F11" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="G11" s="12">
+      <c r="G11" s="18">
         <v>61</v>
       </c>
     </row>
@@ -1230,45 +1265,45 @@
       <c r="A12" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B12" s="13" t="s">
+      <c r="B12" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="C12" s="13" t="s">
+      <c r="C12" s="11" t="s">
         <v>21</v>
       </c>
       <c r="D12" t="s">
         <v>57</v>
       </c>
-      <c r="E12" s="15" t="s">
+      <c r="E12" s="13" t="s">
         <v>59</v>
       </c>
       <c r="F12" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="G12" s="11">
-        <v>60</v>
+      <c r="G12" s="17" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B13" s="13" t="s">
+      <c r="B13" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="C13" s="13" t="s">
+      <c r="C13" s="11" t="s">
         <v>21</v>
       </c>
       <c r="D13" t="s">
         <v>58</v>
       </c>
-      <c r="E13" s="15" t="s">
+      <c r="E13" s="13" t="s">
         <v>59</v>
       </c>
       <c r="F13" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="G13" s="12">
+      <c r="G13" s="18">
         <v>60</v>
       </c>
     </row>
@@ -1276,22 +1311,22 @@
       <c r="A14" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="13" t="s">
+      <c r="B14" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="C14" s="13" t="s">
+      <c r="C14" s="11" t="s">
         <v>19</v>
       </c>
       <c r="D14" t="s">
         <v>60</v>
       </c>
-      <c r="E14" s="15" t="s">
+      <c r="E14" s="13" t="s">
         <v>63</v>
       </c>
       <c r="F14" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="G14" s="11">
+      <c r="G14" s="17">
         <v>62</v>
       </c>
     </row>
@@ -1299,22 +1334,22 @@
       <c r="A15" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B15" s="13" t="s">
+      <c r="B15" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="C15" s="13" t="s">
+      <c r="C15" s="11" t="s">
         <v>19</v>
       </c>
       <c r="D15" t="s">
         <v>61</v>
       </c>
-      <c r="E15" s="15" t="s">
+      <c r="E15" s="13" t="s">
         <v>64</v>
       </c>
       <c r="F15" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="G15" s="12">
+      <c r="G15" s="18">
         <v>64</v>
       </c>
     </row>
@@ -1322,22 +1357,22 @@
       <c r="A16" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B16" s="13" t="s">
+      <c r="B16" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="C16" s="13" t="s">
+      <c r="C16" s="11" t="s">
         <v>19</v>
       </c>
       <c r="D16" t="s">
         <v>62</v>
       </c>
-      <c r="E16" s="15" t="s">
+      <c r="E16" s="13" t="s">
         <v>65</v>
       </c>
       <c r="F16" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="G16" s="11">
+      <c r="G16" s="17">
         <v>66</v>
       </c>
     </row>
@@ -1345,22 +1380,22 @@
       <c r="A17" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B17" s="13" t="s">
+      <c r="B17" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="C17" s="13" t="s">
+      <c r="C17" s="11" t="s">
         <v>19</v>
       </c>
       <c r="D17" t="s">
         <v>66</v>
       </c>
-      <c r="E17" s="15" t="s">
+      <c r="E17" s="13" t="s">
         <v>67</v>
       </c>
       <c r="F17" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="G17" s="12">
+      <c r="G17" s="18">
         <v>61</v>
       </c>
     </row>
@@ -1368,22 +1403,22 @@
       <c r="A18" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B18" s="13" t="s">
+      <c r="B18" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="C18" s="13" t="s">
+      <c r="C18" s="11" t="s">
         <v>68</v>
       </c>
       <c r="D18" t="s">
         <v>69</v>
       </c>
-      <c r="E18" s="15" t="s">
+      <c r="E18" s="13" t="s">
         <v>72</v>
       </c>
       <c r="F18" t="s">
         <v>113</v>
       </c>
-      <c r="G18">
+      <c r="G18" s="19">
         <v>60</v>
       </c>
     </row>
@@ -1391,10 +1426,10 @@
       <c r="A19" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B19" s="13" t="s">
+      <c r="B19" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="C19" s="13" t="s">
+      <c r="C19" s="11" t="s">
         <v>68</v>
       </c>
       <c r="D19" t="s">
@@ -1406,7 +1441,7 @@
       <c r="F19" t="s">
         <v>113</v>
       </c>
-      <c r="G19">
+      <c r="G19" s="19">
         <v>70</v>
       </c>
     </row>
@@ -1414,22 +1449,22 @@
       <c r="A20" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B20" s="13" t="s">
+      <c r="B20" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="C20" s="13" t="s">
+      <c r="C20" s="11" t="s">
         <v>68</v>
       </c>
       <c r="D20" t="s">
         <v>74</v>
       </c>
-      <c r="E20" s="15" t="s">
+      <c r="E20" s="13" t="s">
         <v>73</v>
       </c>
       <c r="F20" t="s">
         <v>113</v>
       </c>
-      <c r="G20">
+      <c r="G20" s="19">
         <v>71</v>
       </c>
     </row>
@@ -1437,22 +1472,22 @@
       <c r="A21" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B21" s="13" t="s">
+      <c r="B21" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="C21" s="13" t="s">
+      <c r="C21" s="11" t="s">
         <v>68</v>
       </c>
       <c r="D21" t="s">
         <v>75</v>
       </c>
-      <c r="E21" s="15" t="s">
+      <c r="E21" s="13" t="s">
         <v>76</v>
       </c>
       <c r="F21" t="s">
         <v>113</v>
       </c>
-      <c r="G21">
+      <c r="G21" s="19">
         <v>73</v>
       </c>
     </row>
@@ -1460,291 +1495,340 @@
       <c r="A22" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B22" s="13" t="s">
+      <c r="B22" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="C22" s="13" t="s">
+      <c r="C22" s="11" t="s">
         <v>68</v>
       </c>
       <c r="D22" t="s">
         <v>78</v>
       </c>
-      <c r="E22" s="15" t="s">
+      <c r="E22" s="13" t="s">
         <v>79</v>
       </c>
       <c r="F22" t="s">
         <v>113</v>
       </c>
-      <c r="G22">
+      <c r="G22" s="19">
         <v>74</v>
       </c>
     </row>
     <row r="23" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="17" t="s">
-        <v>7</v>
-      </c>
-      <c r="B23" s="13" t="s">
+      <c r="A23" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="B23" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="C23" s="13" t="s">
+      <c r="C23" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="D23" s="18"/>
-      <c r="E23" s="18" t="s">
+      <c r="D23" s="16"/>
+      <c r="E23" s="16" t="s">
         <v>117</v>
       </c>
-      <c r="F23" s="18" t="s">
-        <v>124</v>
-      </c>
-      <c r="G23" s="13">
+      <c r="F23" s="16" t="s">
+        <v>123</v>
+      </c>
+      <c r="G23" s="16">
         <v>57</v>
       </c>
       <c r="I23" s="9"/>
     </row>
     <row r="24" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="17" t="s">
-        <v>7</v>
-      </c>
-      <c r="B24" s="13" t="s">
+      <c r="A24" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="B24" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="C24" s="13" t="s">
+      <c r="C24" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="D24" s="18"/>
-      <c r="E24" s="18" t="s">
+      <c r="D24" s="16"/>
+      <c r="E24" s="16" t="s">
+        <v>118</v>
+      </c>
+      <c r="F24" s="16" t="s">
+        <v>137</v>
+      </c>
+      <c r="G24" s="16">
+        <v>58</v>
+      </c>
+      <c r="I24" s="9"/>
+    </row>
+    <row r="25" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="B25" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="C25" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="D25" s="16"/>
+      <c r="E25" s="16" t="s">
         <v>119</v>
       </c>
-      <c r="F24" s="18" t="s">
-        <v>118</v>
-      </c>
-      <c r="G24" s="13">
-        <v>58</v>
-      </c>
-      <c r="I24" s="9"/>
-    </row>
-    <row r="25" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="17" t="s">
-        <v>7</v>
-      </c>
-      <c r="B25" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="C25" s="13" t="s">
+      <c r="F25" s="16" t="s">
+        <v>127</v>
+      </c>
+      <c r="G25" s="16">
+        <v>61</v>
+      </c>
+      <c r="I25" s="9"/>
+    </row>
+    <row r="26" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="B26" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="C26" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="D25" s="18"/>
-      <c r="E25" s="18" t="s">
+      <c r="D26" s="16"/>
+      <c r="E26" s="16" t="s">
         <v>120</v>
       </c>
-      <c r="F25" s="18" t="s">
-        <v>128</v>
-      </c>
-      <c r="G25" s="13">
-        <v>61</v>
-      </c>
-      <c r="I25" s="9"/>
-    </row>
-    <row r="26" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="17" t="s">
-        <v>7</v>
-      </c>
-      <c r="B26" s="13" t="s">
-        <v>83</v>
-      </c>
-      <c r="C26" s="13" t="s">
+      <c r="F26" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="G26" s="16">
+        <v>69</v>
+      </c>
+      <c r="I26" s="9"/>
+    </row>
+    <row r="27" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="B27" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="C27" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="D26" s="18"/>
-      <c r="E26" s="18" t="s">
+      <c r="D27" s="16"/>
+      <c r="E27" s="16" t="s">
         <v>121</v>
       </c>
-      <c r="F26" s="13" t="s">
+      <c r="F27" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="G26" s="13">
-        <v>69</v>
-      </c>
-      <c r="I26" s="9"/>
-    </row>
-    <row r="27" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="17" t="s">
-        <v>7</v>
-      </c>
-      <c r="B27" s="13" t="s">
-        <v>123</v>
-      </c>
-      <c r="C27" s="13" t="s">
+      <c r="G27" s="16">
+        <v>76</v>
+      </c>
+      <c r="I27" s="9"/>
+    </row>
+    <row r="28" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="B28" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="C28" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="D27" s="18"/>
-      <c r="E27" s="18" t="s">
-        <v>122</v>
-      </c>
-      <c r="F27" s="13" t="s">
-        <v>127</v>
-      </c>
-      <c r="G27" s="13">
-        <v>76</v>
-      </c>
-      <c r="I27" s="9"/>
-    </row>
-    <row r="28" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="16" t="s">
-        <v>7</v>
-      </c>
-      <c r="B28" s="13" t="s">
-        <v>84</v>
-      </c>
-      <c r="C28" s="13" t="s">
-        <v>90</v>
-      </c>
-      <c r="E28" s="15" t="s">
+      <c r="E28" s="13" t="s">
         <v>91</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>116</v>
       </c>
+      <c r="G28" s="19" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="29" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="16" t="s">
-        <v>7</v>
-      </c>
-      <c r="B29" s="13" t="s">
+      <c r="A29" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="B29" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="C29" s="13" t="s">
+      <c r="C29" s="11" t="s">
         <v>22</v>
       </c>
       <c r="D29" t="s">
         <v>92</v>
       </c>
-      <c r="E29" s="15" t="s">
+      <c r="E29" s="13" t="s">
         <v>93</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="G29">
+        <v>125</v>
+      </c>
+      <c r="G29" s="19">
         <v>69</v>
       </c>
     </row>
     <row r="30" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="16" t="s">
-        <v>7</v>
-      </c>
-      <c r="B30" s="13" t="s">
+      <c r="A30" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="B30" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="C30" s="13" t="s">
+      <c r="C30" s="11" t="s">
         <v>22</v>
       </c>
       <c r="D30" t="s">
         <v>94</v>
       </c>
-      <c r="E30" s="15" t="s">
+      <c r="E30" s="13" t="s">
         <v>96</v>
       </c>
-      <c r="F30" s="13" t="s">
+      <c r="F30" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="G30" t="s">
+      <c r="G30" s="19" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="31" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="16" t="s">
-        <v>7</v>
-      </c>
-      <c r="B31" s="13" t="s">
+      <c r="A31" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="B31" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="C31" s="13" t="s">
+      <c r="C31" s="11" t="s">
         <v>22</v>
       </c>
       <c r="D31" t="s">
         <v>97</v>
       </c>
-      <c r="E31" s="15" t="s">
+      <c r="E31" s="13" t="s">
         <v>98</v>
       </c>
       <c r="F31" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="G31">
+      <c r="G31" s="19">
         <v>61</v>
       </c>
     </row>
     <row r="32" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="16" t="s">
-        <v>7</v>
-      </c>
-      <c r="B32" s="13" t="s">
+      <c r="A32" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="B32" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="C32" s="13" t="s">
+      <c r="C32" s="11" t="s">
         <v>22</v>
       </c>
       <c r="D32" t="s">
         <v>100</v>
       </c>
-      <c r="E32" s="15" t="s">
+      <c r="E32" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="G32">
+      <c r="F32" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="G32" s="19">
         <v>62</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="16" t="s">
-        <v>7</v>
-      </c>
-      <c r="B33" s="13" t="s">
+      <c r="A33" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="B33" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="C33" s="13" t="s">
+      <c r="C33" s="11" t="s">
         <v>19</v>
       </c>
       <c r="D33" t="s">
         <v>115</v>
       </c>
-      <c r="E33" s="15" t="s">
+      <c r="E33" s="13" t="s">
         <v>99</v>
       </c>
       <c r="F33" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="G33">
+      <c r="G33" s="19">
         <v>68</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="16" t="s">
-        <v>7</v>
-      </c>
-      <c r="B34" s="13" t="s">
+      <c r="A34" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="B34" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="C34" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D34" t="s">
         <v>129</v>
       </c>
-      <c r="C34" s="13" t="s">
+      <c r="E34" s="13" t="s">
+        <v>130</v>
+      </c>
+      <c r="F34" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="G34" s="19">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="B35" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="C35" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="E35" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="F35" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="G35" s="19">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="B36" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="C36" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="D34" t="s">
-        <v>130</v>
-      </c>
-      <c r="E34" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="F34" s="13" t="s">
-        <v>89</v>
-      </c>
-      <c r="G34">
-        <v>81</v>
+      <c r="D36" t="s">
+        <v>139</v>
+      </c>
+      <c r="E36" s="13" t="s">
+        <v>140</v>
+      </c>
+      <c r="F36" t="s">
+        <v>29</v>
+      </c>
+      <c r="G36" s="19" t="s">
+        <v>141</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="3">
     <dataValidation allowBlank="1" showDropDown="1" sqref="E2:E11 G23:G27" xr:uid="{ECD6FAD6-094D-E24F-A15F-528A8178B029}"/>
-    <dataValidation type="list" allowBlank="1" sqref="C2:C11 F30 F9:F10 B11:B22 B28:B34 F34" xr:uid="{9569FF16-2AB7-E348-85C6-E9F1F0C4AAEF}">
+    <dataValidation type="list" allowBlank="1" sqref="C2:C11 F30 F9:F10 B11:B22 B28:B36 F34:F35" xr:uid="{9569FF16-2AB7-E348-85C6-E9F1F0C4AAEF}">
       <formula1>"Layer,Component,Service,Other"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="C23:C27" xr:uid="{5170CA57-58E6-3D47-98DC-4FB63A4BE80D}">
@@ -1759,6 +1843,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6D2115E-F235-624F-B98F-C11728824932}">
   <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="7" max="7" width="10.83203125" style="19"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
@@ -1779,11 +1866,11 @@
       <c r="F1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="20" t="s">
         <v>1</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
@@ -1803,7 +1890,7 @@
         <v>10</v>
       </c>
       <c r="F2" s="9"/>
-      <c r="G2" s="6">
+      <c r="G2" s="7">
         <v>56</v>
       </c>
       <c r="H2" s="9"/>
@@ -1821,11 +1908,11 @@
       <c r="D3" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="14" t="s">
+      <c r="E3" s="12" t="s">
         <v>14</v>
       </c>
       <c r="F3" s="9"/>
-      <c r="G3" s="3">
+      <c r="G3" s="4">
         <v>61</v>
       </c>
       <c r="H3" s="9" t="s">
@@ -1845,11 +1932,11 @@
       <c r="D4" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="14" t="s">
+      <c r="E4" s="12" t="s">
         <v>15</v>
       </c>
       <c r="F4" s="9"/>
-      <c r="G4" s="3">
+      <c r="G4" s="4">
         <v>62</v>
       </c>
       <c r="H4" s="9"/>
@@ -1871,7 +1958,7 @@
         <v>16</v>
       </c>
       <c r="F5" s="9"/>
-      <c r="G5" s="6">
+      <c r="G5" s="7">
         <v>68.69</v>
       </c>
       <c r="H5" s="9"/>
@@ -1893,7 +1980,7 @@
         <v>18</v>
       </c>
       <c r="F6" s="9"/>
-      <c r="G6" s="6">
+      <c r="G6" s="7">
         <v>60</v>
       </c>
       <c r="H6" s="9"/>
@@ -1915,7 +2002,7 @@
         <v>67</v>
       </c>
       <c r="F7" s="9"/>
-      <c r="G7" s="6">
+      <c r="G7" s="7">
         <v>60</v>
       </c>
     </row>

</xml_diff>